<commit_message>
feat: replace fixtures with polished branded ACME documents
Cover sheet with approval stamp, IG Metall contract with CONFIDENTIAL
watermarks and signatures, Outlook-style instructions email, branded
XLSX with revision headers. All numbers verified against source of truth.
</commit_message>
<xml_diff>
--- a/demo/fixtures/acme_q2_2026/demand_forecast_q2.xlsx
+++ b/demo/fixtures/acme_q2_2026/demand_forecast_q2.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,14 +29,40 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="14"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="006A6A6A"/>
+      <sz val="9"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -48,8 +74,18 @@
         <fgColor rgb="001F4E78"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E6DA4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -71,17 +107,91 @@
         <color rgb="00CCCCCC"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="001F4E78"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="001F4E78"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -156,6 +266,149 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="11"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Q2 2026 Demand (tons) by SKU</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Summary'!E3</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Summary'!$A$4:$A$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Summary'!$E$4:$E$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <dLbls>
+          <showVal val="1"/>
+        </dLbls>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>SKU</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Tons</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5040000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -447,218 +700,249 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>sku</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>destination_id</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>city</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>demand_tons</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
+          <t>ACME Logistics GmbH  —  Q2 2026 Demand Forecast  —  Apr</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>Prepared by: S&amp;OP Planning, Munich HQ    •    Revision 3    •    CONFIDENTIAL — Internal Use Only</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>SKU</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Destination ID</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Demand (tons)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
           <t>SKU-001</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>D1</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>Paris</t>
         </is>
       </c>
-      <c r="D2" s="2" t="n">
+      <c r="D4" s="7" t="n">
         <v>56</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>SKU-001</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>D2</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C5" s="10" t="inlineStr">
         <is>
           <t>Vienna</t>
         </is>
       </c>
-      <c r="D3" s="2" t="n">
+      <c r="D5" s="11" t="n">
         <v>49</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>SKU-001</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>D3</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>Amsterdam</t>
         </is>
       </c>
-      <c r="D4" s="2" t="n">
+      <c r="D6" s="7" t="n">
         <v>35</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>SKU-002</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>D1</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C7" s="10" t="inlineStr">
         <is>
           <t>Paris</t>
         </is>
       </c>
-      <c r="D5" s="2" t="n">
+      <c r="D7" s="11" t="n">
         <v>46</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>SKU-002</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>D2</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>Vienna</t>
         </is>
       </c>
-      <c r="D6" s="2" t="n">
+      <c r="D8" s="7" t="n">
         <v>40.25</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>SKU-002</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>D3</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C9" s="10" t="inlineStr">
         <is>
           <t>Amsterdam</t>
         </is>
       </c>
-      <c r="D7" s="2" t="n">
+      <c r="D9" s="11" t="n">
         <v>28.75</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>SKU-003</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>D1</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>Paris</t>
         </is>
       </c>
-      <c r="D8" s="2" t="n">
+      <c r="D10" s="7" t="n">
         <v>50</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>SKU-003</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>D2</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C11" s="10" t="inlineStr">
         <is>
           <t>Vienna</t>
         </is>
       </c>
-      <c r="D9" s="2" t="n">
+      <c r="D11" s="11" t="n">
         <v>43.75</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>SKU-003</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>D3</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>Amsterdam</t>
         </is>
       </c>
-      <c r="D10" s="2" t="n">
+      <c r="D12" s="7" t="n">
         <v>31.25</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>TOTAL Apr</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="n"/>
+      <c r="C13" s="13" t="n"/>
+      <c r="D13" s="14" t="n">
+        <v>380</v>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -669,218 +953,249 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>sku</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>destination_id</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>city</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>demand_tons</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
+          <t>ACME Logistics GmbH  —  Q2 2026 Demand Forecast  —  May</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>Prepared by: S&amp;OP Planning, Munich HQ    •    Revision 3    •    CONFIDENTIAL — Internal Use Only</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>SKU</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Destination ID</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Demand (tons)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
           <t>SKU-001</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>D1</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>Paris</t>
         </is>
       </c>
-      <c r="D2" s="2" t="n">
+      <c r="D4" s="7" t="n">
         <v>62</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>SKU-001</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>D2</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C5" s="10" t="inlineStr">
         <is>
           <t>Vienna</t>
         </is>
       </c>
-      <c r="D3" s="2" t="n">
+      <c r="D5" s="11" t="n">
         <v>54.25</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>SKU-001</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>D3</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>Amsterdam</t>
         </is>
       </c>
-      <c r="D4" s="2" t="n">
+      <c r="D6" s="7" t="n">
         <v>38.75</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>SKU-002</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>D1</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C7" s="10" t="inlineStr">
         <is>
           <t>Paris</t>
         </is>
       </c>
-      <c r="D5" s="2" t="n">
+      <c r="D7" s="11" t="n">
         <v>48</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>SKU-002</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>D2</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>Vienna</t>
         </is>
       </c>
-      <c r="D6" s="2" t="n">
+      <c r="D8" s="7" t="n">
         <v>42</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>SKU-002</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>D3</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C9" s="10" t="inlineStr">
         <is>
           <t>Amsterdam</t>
         </is>
       </c>
-      <c r="D7" s="2" t="n">
+      <c r="D9" s="11" t="n">
         <v>30</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>SKU-003</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>D1</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>Paris</t>
         </is>
       </c>
-      <c r="D8" s="2" t="n">
+      <c r="D10" s="7" t="n">
         <v>54</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>SKU-003</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>D2</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C11" s="10" t="inlineStr">
         <is>
           <t>Vienna</t>
         </is>
       </c>
-      <c r="D9" s="2" t="n">
+      <c r="D11" s="11" t="n">
         <v>47.25</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>SKU-003</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>D3</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>Amsterdam</t>
         </is>
       </c>
-      <c r="D10" s="2" t="n">
+      <c r="D12" s="7" t="n">
         <v>33.75</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>TOTAL May</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="n"/>
+      <c r="C13" s="13" t="n"/>
+      <c r="D13" s="14" t="n">
+        <v>410</v>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -891,218 +1206,249 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>sku</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>destination_id</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>city</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>demand_tons</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
+          <t>ACME Logistics GmbH  —  Q2 2026 Demand Forecast  —  Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>Prepared by: S&amp;OP Planning, Munich HQ    •    Revision 3    •    CONFIDENTIAL — Internal Use Only</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>SKU</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Destination ID</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Demand (tons)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
           <t>SKU-001</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>D1</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>Paris</t>
         </is>
       </c>
-      <c r="D2" s="2" t="n">
+      <c r="D4" s="7" t="n">
         <v>64</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>SKU-001</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>D2</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C5" s="10" t="inlineStr">
         <is>
           <t>Vienna</t>
         </is>
       </c>
-      <c r="D3" s="2" t="n">
+      <c r="D5" s="11" t="n">
         <v>56</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>SKU-001</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>D3</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>Amsterdam</t>
         </is>
       </c>
-      <c r="D4" s="2" t="n">
+      <c r="D6" s="7" t="n">
         <v>40</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>SKU-002</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>D1</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C7" s="10" t="inlineStr">
         <is>
           <t>Paris</t>
         </is>
       </c>
-      <c r="D5" s="2" t="n">
+      <c r="D7" s="11" t="n">
         <v>50</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>SKU-002</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>D2</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>Vienna</t>
         </is>
       </c>
-      <c r="D6" s="2" t="n">
+      <c r="D8" s="7" t="n">
         <v>43.75</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>SKU-002</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>D3</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C9" s="10" t="inlineStr">
         <is>
           <t>Amsterdam</t>
         </is>
       </c>
-      <c r="D7" s="2" t="n">
+      <c r="D9" s="11" t="n">
         <v>31.25</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>SKU-003</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>D1</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>Paris</t>
         </is>
       </c>
-      <c r="D8" s="2" t="n">
+      <c r="D10" s="7" t="n">
         <v>53.2</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>SKU-003</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>D2</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C11" s="10" t="inlineStr">
         <is>
           <t>Vienna</t>
         </is>
       </c>
-      <c r="D9" s="2" t="n">
+      <c r="D11" s="11" t="n">
         <v>46.55</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>SKU-003</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>D3</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>Amsterdam</t>
         </is>
       </c>
-      <c r="D10" s="2" t="n">
+      <c r="D12" s="7" t="n">
         <v>33.25</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>TOTAL Jun</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="n"/>
+      <c r="C13" s="13" t="n"/>
+      <c r="D13" s="14" t="n">
+        <v>418</v>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1113,7 +1459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1121,112 +1467,168 @@
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="56" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>sku</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
+          <t>ACME Logistics GmbH  —  Q2 2026 Demand Forecast  —  Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Prepared by: S&amp;OP Planning, Munich HQ    •    Revision 3    •    CONFIDENTIAL — Internal Use Only</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>SKU</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Apr</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>May</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Jun</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Q2_total</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Q2 Total</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>SKU-001</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n">
+      <c r="B4" s="15" t="n">
         <v>140</v>
       </c>
-      <c r="C2" s="2" t="n">
+      <c r="C4" s="15" t="n">
         <v>155</v>
       </c>
-      <c r="D2" s="2" t="n">
+      <c r="D4" s="15" t="n">
         <v>160</v>
       </c>
-      <c r="E2" s="2" t="n">
-        <v>455</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="E4" s="16">
+        <f>SUM(B4:D4)</f>
+        <v/>
+      </c>
+      <c r="F4" s="17" t="inlineStr">
+        <is>
+          <t>Focus item — Munich preferred routing where cost-effective</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>SKU-002</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n">
+      <c r="B5" s="18" t="n">
         <v>115</v>
       </c>
-      <c r="C3" s="2" t="n">
+      <c r="C5" s="18" t="n">
         <v>120</v>
       </c>
-      <c r="D3" s="2" t="n">
+      <c r="D5" s="18" t="n">
         <v>125</v>
       </c>
-      <c r="E3" s="2" t="n">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="E5" s="19">
+        <f>SUM(B5:D5)</f>
+        <v/>
+      </c>
+      <c r="F5" s="20" t="inlineStr">
+        <is>
+          <t>Standard distribution — maintain current warehouse mix</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>SKU-003</t>
         </is>
       </c>
-      <c r="B4" s="2" t="n">
+      <c r="B6" s="15" t="n">
         <v>125</v>
       </c>
-      <c r="C4" s="2" t="n">
+      <c r="C6" s="15" t="n">
         <v>135</v>
       </c>
-      <c r="D4" s="2" t="n">
+      <c r="D6" s="15" t="n">
         <v>133</v>
       </c>
-      <c r="E4" s="2" t="n">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="E6" s="16">
+        <f>SUM(B6:D6)</f>
+        <v/>
+      </c>
+      <c r="F6" s="17" t="inlineStr">
+        <is>
+          <t>Standard distribution — monitor Hamburg capacity</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B5" s="2" t="n">
-        <v>380</v>
-      </c>
-      <c r="C5" s="2" t="n">
-        <v>410</v>
-      </c>
-      <c r="D5" s="2" t="n">
-        <v>418</v>
-      </c>
-      <c r="E5" s="2" t="n">
-        <v>1208</v>
+      <c r="B7" s="21">
+        <f>SUM(B4:B6)</f>
+        <v/>
+      </c>
+      <c r="C7" s="21">
+        <f>SUM(C4:C6)</f>
+        <v/>
+      </c>
+      <c r="D7" s="21">
+        <f>SUM(D4:D6)</f>
+        <v/>
+      </c>
+      <c r="E7" s="21">
+        <f>SUM(E4:E6)</f>
+        <v/>
+      </c>
+      <c r="F7" s="22" t="inlineStr"/>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="23" t="inlineStr">
+        <is>
+          <t>Source: ACME S&amp;OP consensus forecast, approved 17 Apr 2026  |  Forecast horizon: 1 Apr – 30 Jun 2026  |  Destination split: D1 Paris 40%, D2 Vienna 35%, D3 Amsterdam 25%  |  Document ID: SOP-Q2-2026-R3</t>
+        </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A10:F10"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>